<commit_message>
#1 #2 Heat sink updated in schematic and BOM file. PDF updated.
</commit_message>
<xml_diff>
--- a/Design-Files/Power-Switcher-v1.0/Deliverables/BOM/Power-Switcher-v1.0.xlsx
+++ b/Design-Files/Power-Switcher-v1.0/Deliverables/BOM/Power-Switcher-v1.0.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28925"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\stephen-autoPWRswitcher\Design-Files\Power-Switcher-v1.0\Deliverables\BOM\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{154059AB-19FF-4193-B12B-79C052A8C093}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView windowWidth="20490" windowHeight="7620"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,8 +24,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -275,29 +279,23 @@
     <t>HeatSink</t>
   </si>
   <si>
-    <t xml:space="preserve">30*30*10MM 6063-T5 aluminum Heat sink / cooling fin </t>
-  </si>
-  <si>
     <t>Custom</t>
   </si>
   <si>
-    <t>XSDJ7-122</t>
-  </si>
-  <si>
     <t>XSD</t>
+  </si>
+  <si>
+    <t>XSD183-097-B</t>
+  </si>
+  <si>
+    <t>31.3*18.5*45MM 6063-T5 Heat sink / cooling fin ROHS</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-  </numFmts>
-  <fonts count="25">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -340,152 +338,8 @@
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="35">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -504,194 +358,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="16">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -782,251 +450,9 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="49">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
   <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -1069,67 +495,23 @@
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="49">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Currency" xfId="2" builtinId="4"/>
-    <cellStyle name="Percent" xfId="3" builtinId="5"/>
-    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
-    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
-    <cellStyle name="Hyperlink" xfId="6" builtinId="8"/>
-    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
-    <cellStyle name="Note" xfId="8" builtinId="10"/>
-    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
-    <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
-    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
-    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
-    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
-    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
-    <cellStyle name="Input" xfId="16" builtinId="20"/>
-    <cellStyle name="Output" xfId="17" builtinId="21"/>
-    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
-    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
-    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
-    <cellStyle name="Total" xfId="21" builtinId="25"/>
-    <cellStyle name="Good" xfId="22" builtinId="26"/>
-    <cellStyle name="Bad" xfId="23" builtinId="27"/>
-    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
-    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
-    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
-    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
-    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
-    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
-    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
-      <color rgb="0003A4CB"/>
-      <color rgb="002CD0B2"/>
+      <color rgb="FF03A4CB"/>
+      <color rgb="FF2CD0B2"/>
     </mruColors>
   </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1387,28 +769,29 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:K16"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="3.14285714285714" style="1" customWidth="1"/>
-    <col min="3" max="3" width="18.7142857142857" style="1" customWidth="1"/>
+    <col min="2" max="2" width="3.140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="18.7109375" style="1" customWidth="1"/>
     <col min="4" max="4" width="36" customWidth="1"/>
     <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="15.1428571428571" customWidth="1"/>
-    <col min="7" max="7" width="33.4285714285714" customWidth="1"/>
-    <col min="8" max="8" width="21.4285714285714" customWidth="1"/>
-    <col min="9" max="9" width="6.71428571428571" customWidth="1"/>
-    <col min="10" max="10" width="9.28571428571429" customWidth="1"/>
-    <col min="11" max="11" width="9.14285714285714" customWidth="1"/>
+    <col min="6" max="6" width="15.140625" customWidth="1"/>
+    <col min="7" max="7" width="33.42578125" customWidth="1"/>
+    <col min="8" max="8" width="21.42578125" customWidth="1"/>
+    <col min="9" max="9" width="6.7109375" customWidth="1"/>
+    <col min="10" max="10" width="9.28515625" customWidth="1"/>
+    <col min="11" max="11" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" spans="1:11">
+    <row r="1" spans="1:11">
       <c r="A1" s="2"/>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -1421,7 +804,7 @@
       <c r="J1" s="14"/>
       <c r="K1" s="14"/>
     </row>
-    <row r="2" ht="15.75" spans="1:11">
+    <row r="2" spans="1:11">
       <c r="A2" s="2"/>
       <c r="B2" s="5" t="s">
         <v>0</v>
@@ -1454,10 +837,10 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" ht="15.75" spans="1:11">
+    <row r="3" spans="1:11">
       <c r="A3" s="2"/>
       <c r="B3" s="7">
-        <f>ROW(B3)-ROW($B$2)</f>
+        <f t="shared" ref="B3:B16" si="0">ROW(B3)-ROW($B$2)</f>
         <v>1</v>
       </c>
       <c r="C3" s="8" t="s">
@@ -1486,10 +869,10 @@
       </c>
       <c r="K3" s="9"/>
     </row>
-    <row r="4" ht="15.75" spans="1:11">
+    <row r="4" spans="1:11">
       <c r="A4" s="2"/>
       <c r="B4" s="7">
-        <f>ROW(B4)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="C4" s="11" t="s">
@@ -1518,10 +901,10 @@
       </c>
       <c r="K4" s="12"/>
     </row>
-    <row r="5" ht="15.75" spans="1:11">
+    <row r="5" spans="1:11">
       <c r="A5" s="2"/>
       <c r="B5" s="7">
-        <f>ROW(B5)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="C5" s="8" t="s">
@@ -1550,10 +933,10 @@
       </c>
       <c r="K5" s="9"/>
     </row>
-    <row r="6" ht="15.75" spans="1:11">
+    <row r="6" spans="1:11" ht="24">
       <c r="A6" s="2"/>
       <c r="B6" s="7">
-        <f>ROW(B6)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="C6" s="11" t="s">
@@ -1582,10 +965,10 @@
       </c>
       <c r="K6" s="12"/>
     </row>
-    <row r="7" ht="15.75" spans="1:11">
+    <row r="7" spans="1:11">
       <c r="A7" s="2"/>
       <c r="B7" s="7">
-        <f>ROW(B7)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="C7" s="8" t="s">
@@ -1614,10 +997,10 @@
       </c>
       <c r="K7" s="9"/>
     </row>
-    <row r="8" ht="48.75" spans="1:11">
+    <row r="8" spans="1:11" ht="48">
       <c r="A8" s="2"/>
       <c r="B8" s="7">
-        <f>ROW(B8)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="C8" s="11" t="s">
@@ -1646,10 +1029,10 @@
       </c>
       <c r="K8" s="12"/>
     </row>
-    <row r="9" ht="24.75" spans="1:11">
+    <row r="9" spans="1:11" ht="24">
       <c r="A9" s="2"/>
       <c r="B9" s="7">
-        <f>ROW(B9)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="C9" s="8" t="s">
@@ -1678,10 +1061,10 @@
       </c>
       <c r="K9" s="9"/>
     </row>
-    <row r="10" ht="15.75" spans="1:11">
+    <row r="10" spans="1:11">
       <c r="A10" s="2"/>
       <c r="B10" s="7">
-        <f>ROW(B10)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="C10" s="11" t="s">
@@ -1710,10 +1093,10 @@
       </c>
       <c r="K10" s="12"/>
     </row>
-    <row r="11" ht="15.75" spans="1:11">
+    <row r="11" spans="1:11">
       <c r="A11" s="2"/>
       <c r="B11" s="7">
-        <f>ROW(B11)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>9</v>
       </c>
       <c r="C11" s="8" t="s">
@@ -1742,10 +1125,10 @@
       </c>
       <c r="K11" s="9"/>
     </row>
-    <row r="12" ht="15.75" spans="1:11">
+    <row r="12" spans="1:11">
       <c r="A12" s="2"/>
       <c r="B12" s="7">
-        <f>ROW(B12)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="C12" s="11" t="s">
@@ -1774,10 +1157,10 @@
       </c>
       <c r="K12" s="12"/>
     </row>
-    <row r="13" ht="15.75" spans="1:11">
+    <row r="13" spans="1:11">
       <c r="A13" s="2"/>
       <c r="B13" s="7">
-        <f>ROW(B13)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
       <c r="C13" s="8" t="s">
@@ -1806,10 +1189,10 @@
       </c>
       <c r="K13" s="9"/>
     </row>
-    <row r="14" ht="15.75" spans="1:11">
+    <row r="14" spans="1:11">
       <c r="A14" s="2"/>
       <c r="B14" s="7">
-        <f>ROW(B14)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
       <c r="C14" s="11" t="s">
@@ -1838,10 +1221,10 @@
       </c>
       <c r="K14" s="12"/>
     </row>
-    <row r="15" ht="24.75" spans="1:11">
+    <row r="15" spans="1:11" ht="24">
       <c r="A15" s="2"/>
       <c r="B15" s="7">
-        <f>ROW(B15)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>13</v>
       </c>
       <c r="C15" s="8" t="s">
@@ -1870,9 +1253,9 @@
       </c>
       <c r="K15" s="9"/>
     </row>
-    <row r="16" ht="24.75" spans="2:11">
+    <row r="16" spans="1:11" ht="24">
       <c r="B16" s="7">
-        <f>ROW(B16)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>14</v>
       </c>
       <c r="C16" s="8" t="s">
@@ -1882,22 +1265,22 @@
         <v>81</v>
       </c>
       <c r="E16" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="F16" s="9" t="s">
         <v>82</v>
-      </c>
-      <c r="F16" s="9" t="s">
-        <v>83</v>
       </c>
       <c r="G16" s="10" t="s">
         <v>84</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="I16" s="10" t="s">
         <v>28</v>
       </c>
       <c r="J16" s="9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K16" s="9"/>
     </row>
@@ -1907,6 +1290,5 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
-  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>